<commit_message>
made changes for LAHSA
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\Automation projects\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Product\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B45333E3-697A-4E2F-86DC-2EA558FA1E0F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F5CA9D9-5112-485B-B073-07E31699D469}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4097" yWindow="1029" windowWidth="16457" windowHeight="8554" firstSheet="6" activeTab="7" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="7" activeTab="7" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="90">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -121,15 +121,6 @@
     <t>GranteeMatch__c</t>
   </si>
   <si>
-    <t>QSubmissionDeadline__c</t>
-  </si>
-  <si>
-    <t>AResponseDeadline__c</t>
-  </si>
-  <si>
-    <t>QAContactEmailAddress__c</t>
-  </si>
-  <si>
     <t>AwardFloor__c</t>
   </si>
   <si>
@@ -248,13 +239,94 @@
   </si>
   <si>
     <t>Automation Runtime Competitive Past Announcement</t>
+  </si>
+  <si>
+    <t>fieldAnnouncementName__c</t>
+  </si>
+  <si>
+    <t>fieldProgram__c</t>
+  </si>
+  <si>
+    <t>fieldBudget_Category_Package__c</t>
+  </si>
+  <si>
+    <t>fieldIsMatchRequired__c</t>
+  </si>
+  <si>
+    <t>fieldLaverageAllowed__c</t>
+  </si>
+  <si>
+    <t>fieldIsProgramIncomeAnticipated__c</t>
+  </si>
+  <si>
+    <t>fieldPreApplicationNeeded__c</t>
+  </si>
+  <si>
+    <t>fieldFocusAreaRequired__c</t>
+  </si>
+  <si>
+    <t>fieldKPIsRequired__c</t>
+  </si>
+  <si>
+    <t>fieldWBSRequired__c</t>
+  </si>
+  <si>
+    <t>fieldRiskAssessment_Required__c</t>
+  </si>
+  <si>
+    <t>fieldAreExpensesBuildIUpLevel__c</t>
+  </si>
+  <si>
+    <t>fieldIsAdvancePermitted__c</t>
+  </si>
+  <si>
+    <t>fieldIsNegotiationsAllowed__c</t>
+  </si>
+  <si>
+    <t>fieldGranteeMatch__c</t>
+  </si>
+  <si>
+    <t>fieldIsGoalsRequired__c</t>
+  </si>
+  <si>
+    <t>fieldAnnouncementDescription__c</t>
+  </si>
+  <si>
+    <t>fieldEligibleApplicantTypes__c</t>
+  </si>
+  <si>
+    <t>fieldApplicationDueDate__c</t>
+  </si>
+  <si>
+    <t>fieldQAAvailability__c</t>
+  </si>
+  <si>
+    <t>fieldQSubmissionDeadline__c</t>
+  </si>
+  <si>
+    <t>fieldAResponseDeadline__c</t>
+  </si>
+  <si>
+    <t>fieldQAContactEmailAddress__c</t>
+  </si>
+  <si>
+    <t>fieldAwardFloor__c</t>
+  </si>
+  <si>
+    <t>fieldAwardCeiling__c</t>
+  </si>
+  <si>
+    <t>fieldEstimatedNumberOfAwards__c</t>
+  </si>
+  <si>
+    <t>fieldTotalCommittedAmount__c</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -284,6 +356,12 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF222222"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -306,7 +384,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -319,6 +397,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -635,14 +714,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE354EA7-EF61-4CF6-8FD9-4C0F8CF01A30}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.4609375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.3046875" customWidth="1"/>
-    <col min="3" max="3" width="43.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -653,40 +732,40 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>63</v>
       </c>
       <c r="C2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
       <c r="C3" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>65</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C12" s="5"/>
     </row>
   </sheetData>
@@ -698,14 +777,14 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5419849D-2139-4751-9485-A00468AD6907}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.69140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -716,128 +795,128 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
-        <v>13</v>
+      <c r="B2" s="6" t="s">
+        <v>79</v>
       </c>
       <c r="C2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>80</v>
       </c>
       <c r="C3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>81</v>
       </c>
       <c r="C4">
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>82</v>
       </c>
       <c r="C5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="C6">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>84</v>
       </c>
       <c r="C7">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>86</v>
       </c>
       <c r="C9">
         <v>1000</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>87</v>
       </c>
       <c r="C10">
         <v>10000</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>88</v>
       </c>
       <c r="C11">
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>89</v>
       </c>
       <c r="C12">
         <v>10000</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="G13">
         <v>0</v>
       </c>
@@ -853,14 +932,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FF67A45-0B54-4944-9B39-F82B26EF60B6}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.69140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -871,7 +950,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -882,7 +961,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -890,10 +969,10 @@
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -904,7 +983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -912,21 +991,21 @@
         <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C6">
         <v>1000</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -937,18 +1016,18 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C8">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -967,13 +1046,13 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F105F821-5E53-4FD8-9F07-CF97205700C1}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -984,7 +1063,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -995,7 +1074,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1003,10 +1082,10 @@
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1017,29 +1096,29 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C5">
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C6">
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1047,21 +1126,21 @@
         <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C8">
         <v>1000</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1072,18 +1151,18 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C10">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -1103,13 +1182,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC101BFC-1550-4137-B012-E4749B310065}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1120,7 +1199,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1131,7 +1210,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1139,10 +1218,10 @@
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1153,29 +1232,29 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C5">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C6">
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1183,21 +1262,21 @@
         <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C8">
         <v>1000</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1208,18 +1287,18 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C10">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -1238,14 +1317,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896B5C7-9641-468E-8213-95D0BE0FBE7C}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.4609375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.69140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1256,23 +1335,23 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C2">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C3">
         <v>379</v>
@@ -1286,13 +1365,13 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="20.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.69140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1303,59 +1382,59 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
         <v>32</v>
       </c>
-      <c r="C2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="C4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C5">
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -1367,13 +1446,13 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B029D8-A57A-4DED-8831-111F395CEFC2}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1384,147 +1463,147 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
-        <v>9</v>
+      <c r="B2" s="6" t="s">
+        <v>66</v>
       </c>
       <c r="C2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
-        <v>22</v>
+      <c r="B3" s="6" t="s">
+        <v>77</v>
       </c>
       <c r="C3">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
-        <v>10</v>
+      <c r="B4" s="6" t="s">
+        <v>67</v>
       </c>
       <c r="C4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" t="s">
-        <v>11</v>
+      <c r="B5" s="6" t="s">
+        <v>68</v>
       </c>
       <c r="C5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
-      <c r="B6" t="s">
-        <v>12</v>
+      <c r="B6" s="6" t="s">
+        <v>69</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
-      <c r="B7" t="s">
-        <v>39</v>
+      <c r="B7" s="6" t="s">
+        <v>72</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
-      <c r="B8" t="s">
-        <v>37</v>
+      <c r="B8" s="6" t="s">
+        <v>73</v>
       </c>
       <c r="C8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
-      <c r="B9" t="s">
-        <v>41</v>
+      <c r="B9" s="6" t="s">
+        <v>70</v>
       </c>
       <c r="C9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
+        <v>78</v>
       </c>
       <c r="C10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>3</v>
       </c>
-      <c r="B11" t="s">
-        <v>43</v>
+      <c r="B11" s="6" t="s">
+        <v>71</v>
       </c>
       <c r="C11" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>3</v>
       </c>
-      <c r="B12" t="s">
-        <v>40</v>
+      <c r="B12" s="6" t="s">
+        <v>74</v>
       </c>
       <c r="C12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>3</v>
       </c>
-      <c r="B13" t="s">
-        <v>44</v>
+      <c r="B13" s="6" t="s">
+        <v>75</v>
       </c>
       <c r="C13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
-      <c r="B14" t="s">
-        <v>45</v>
+      <c r="B14" s="6" t="s">
+        <v>76</v>
       </c>
       <c r="C14" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -1536,13 +1615,13 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A5EA066-8BD7-4F60-A549-8DF4B566C85E}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1553,7 +1632,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1561,10 +1640,10 @@
         <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1572,10 +1651,10 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1583,10 +1662,10 @@
         <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1594,95 +1673,95 @@
         <v>12</v>
       </c>
       <c r="C5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
         <v>39</v>
       </c>
-      <c r="C6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
         <v>37</v>
       </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
         <v>41</v>
       </c>
-      <c r="C8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
         <v>42</v>
       </c>
-      <c r="C9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>45</v>
-      </c>
       <c r="C13" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -1693,13 +1772,13 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68EBF6E6-8687-4CE1-8BB6-330DEC350611}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1710,7 +1789,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1721,7 +1800,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1732,7 +1811,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1743,7 +1822,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1754,7 +1833,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1762,95 +1841,95 @@
         <v>12</v>
       </c>
       <c r="C6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
         <v>39</v>
       </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
         <v>37</v>
       </c>
-      <c r="C8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
         <v>41</v>
       </c>
-      <c r="C9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
         <v>42</v>
       </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>45</v>
-      </c>
       <c r="C14" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -1861,13 +1940,13 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B71B207-7F71-4F84-BC32-C3056B8DABA1}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1878,7 +1957,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1889,7 +1968,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1900,7 +1979,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1911,7 +1990,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1922,7 +2001,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1933,92 +2012,92 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
       <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
         <v>39</v>
       </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
         <v>37</v>
       </c>
-      <c r="C8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
         <v>41</v>
       </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
         <v>42</v>
       </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>45</v>
-      </c>
       <c r="C14" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -2029,14 +2108,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FC5EB7D-13BF-4B5E-895C-F5B651828B55}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.4609375" customWidth="1"/>
-    <col min="2" max="2" width="26.3046875" customWidth="1"/>
-    <col min="3" max="3" width="62.23046875" customWidth="1"/>
+    <col min="1" max="1" width="30.42578125" customWidth="1"/>
+    <col min="2" max="2" width="26.28515625" customWidth="1"/>
+    <col min="3" max="3" width="62.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2047,7 +2126,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2055,10 +2134,10 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2066,10 +2145,10 @@
         <v>5</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2077,7 +2156,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -2088,14 +2167,14 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFE25EE6-66F5-4951-9D0C-F6559D035D9C}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.53515625" customWidth="1"/>
-    <col min="2" max="2" width="31.69140625" customWidth="1"/>
-    <col min="3" max="3" width="14.07421875" customWidth="1"/>
+    <col min="1" max="1" width="14.5703125" customWidth="1"/>
+    <col min="2" max="2" width="31.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2106,7 +2185,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2117,7 +2196,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2128,7 +2207,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2139,7 +2218,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2150,92 +2229,92 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
       <c r="B6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
         <v>39</v>
       </c>
-      <c r="C6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
         <v>37</v>
       </c>
-      <c r="C7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
         <v>41</v>
       </c>
-      <c r="C8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
         <v>42</v>
       </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>45</v>
-      </c>
       <c r="C13" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -2246,14 +2325,14 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B83C7FC7-2A18-436E-A373-D289D769241C}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.53515625" customWidth="1"/>
-    <col min="2" max="2" width="24.4609375" customWidth="1"/>
-    <col min="3" max="3" width="15.69140625" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" customWidth="1"/>
+    <col min="2" max="2" width="24.42578125" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2264,7 +2343,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2275,7 +2354,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2286,7 +2365,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2297,7 +2376,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2308,7 +2387,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2319,92 +2398,92 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
       <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
         <v>39</v>
       </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
         <v>37</v>
       </c>
-      <c r="C8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
         <v>41</v>
       </c>
-      <c r="C9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
         <v>42</v>
       </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>45</v>
-      </c>
       <c r="C14" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -2415,13 +2494,13 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{471A3BD1-3EAB-4C67-9345-90730B6A7403}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2432,7 +2511,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2443,7 +2522,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2454,7 +2533,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2465,7 +2544,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2476,7 +2555,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2487,92 +2566,92 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
       <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
         <v>39</v>
       </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
         <v>37</v>
       </c>
-      <c r="C8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
         <v>41</v>
       </c>
-      <c r="C9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
         <v>42</v>
       </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>45</v>
-      </c>
       <c r="C14" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -2583,13 +2662,13 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A836B93B-2094-42BE-9D92-A2EB5434CB28}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.07421875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.69140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2600,26 +2679,26 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" t="s">
         <v>47</v>
-      </c>
-      <c r="C2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C3" t="s">
-        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -2631,13 +2710,13 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB402F88-9436-4279-8D3B-028474BBC575}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.4609375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2648,7 +2727,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2659,7 +2738,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2670,7 +2749,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2681,7 +2760,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2692,7 +2771,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2703,92 +2782,92 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
       <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
         <v>39</v>
       </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
         <v>37</v>
       </c>
-      <c r="C8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
         <v>41</v>
       </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
         <v>42</v>
       </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>45</v>
-      </c>
       <c r="C14" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -2799,14 +2878,14 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61C91C76-2A92-4FAB-8589-A8F89F7DC3A0}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.69140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2817,18 +2896,18 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>19</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C9" s="3"/>
     </row>
   </sheetData>
@@ -2839,14 +2918,14 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF72FB96-7C2F-4711-BDC9-46D87BC44E74}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.4609375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.3046875" customWidth="1"/>
-    <col min="3" max="3" width="43.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2857,7 +2936,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2868,7 +2947,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2879,7 +2958,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2890,7 +2969,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2901,7 +2980,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2909,95 +2988,95 @@
         <v>12</v>
       </c>
       <c r="C6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
         <v>39</v>
       </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
         <v>37</v>
       </c>
-      <c r="C8" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
         <v>41</v>
       </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
         <v>42</v>
       </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>45</v>
-      </c>
       <c r="C14" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -3008,14 +3087,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9C8260A-2B08-45B2-91C9-3D139644FA31}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.4609375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.3046875" customWidth="1"/>
-    <col min="3" max="3" width="59.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="59.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3026,40 +3105,40 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
-        <v>4</v>
+      <c r="B2" s="6" t="s">
+        <v>63</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
-        <v>5</v>
+      <c r="B3" s="6" t="s">
+        <v>64</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
-        <v>6</v>
+      <c r="B4" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C9" s="5"/>
     </row>
   </sheetData>
@@ -3071,14 +3150,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{801045D0-434D-4772-B50B-BAD32ADFCC6D}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33.84375" customWidth="1"/>
-    <col min="2" max="2" width="30.07421875" customWidth="1"/>
+    <col min="1" max="1" width="33.85546875" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" customWidth="1"/>
     <col min="3" max="3" width="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3089,7 +3168,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3097,10 +3176,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3108,10 +3187,10 @@
         <v>5</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -3130,13 +3209,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{312DC3EE-E575-46F9-A9B5-EB471905BC17}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="29.4609375" customWidth="1"/>
-    <col min="3" max="3" width="65.84375" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" customWidth="1"/>
+    <col min="3" max="3" width="65.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3147,7 +3226,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3155,10 +3234,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3166,10 +3245,10 @@
         <v>5</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -3189,13 +3268,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{628A250B-2421-4501-B6A1-3551362D1E63}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="31.3046875" customWidth="1"/>
-    <col min="3" max="3" width="46.53515625" customWidth="1"/>
+    <col min="2" max="2" width="31.28515625" customWidth="1"/>
+    <col min="3" max="3" width="46.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3206,7 +3285,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3214,10 +3293,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3225,10 +3304,10 @@
         <v>5</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -3247,13 +3326,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67385A93-9DB4-418E-B977-B594C234D617}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="44.69140625" customWidth="1"/>
-    <col min="3" max="3" width="38.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="44.7109375" customWidth="1"/>
+    <col min="3" max="3" width="38.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3264,7 +3343,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3272,10 +3351,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3283,10 +3362,10 @@
         <v>5</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -3306,14 +3385,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C81AF588-AABE-4434-A649-BE45CA5F0598}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.4609375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.3046875" customWidth="1"/>
-    <col min="3" max="3" width="43.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3324,34 +3403,34 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
-        <v>4</v>
+      <c r="B2" s="6" t="s">
+        <v>63</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>64</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>65</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
@@ -3366,14 +3445,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F5A36B1-BCE1-494C-9FF2-9E81EB69D145}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.4609375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.3046875" customWidth="1"/>
-    <col min="3" max="3" width="43.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3384,7 +3463,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3392,10 +3471,10 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3403,10 +3482,10 @@
         <v>5</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
made changes in the sanity , execl sheet and payloads
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Product\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F5CA9D9-5112-485B-B073-07E31699D469}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA99C194-925D-4A2D-9E1F-8ED92169490D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="7" activeTab="7" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="13" activeTab="16" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -29,16 +29,17 @@
     <sheet name="BudgetPeriod" sheetId="3" r:id="rId14"/>
     <sheet name="Reviewer" sheetId="4" r:id="rId15"/>
     <sheet name="Creation Second Modal" sheetId="6" r:id="rId16"/>
-    <sheet name="Creation Second Modal for App" sheetId="25" r:id="rId17"/>
-    <sheet name="Creation Second Modal FA" sheetId="24" r:id="rId18"/>
-    <sheet name="Creation Second Modal1" sheetId="14" r:id="rId19"/>
-    <sheet name="Creation Second Modal3" sheetId="17" r:id="rId20"/>
-    <sheet name="Creation Second Modal4" sheetId="18" r:id="rId21"/>
-    <sheet name="Creation of Second Modal" sheetId="15" r:id="rId22"/>
-    <sheet name="EnterReview" sheetId="9" r:id="rId23"/>
-    <sheet name="Pre-Application Modal" sheetId="11" r:id="rId24"/>
-    <sheet name="Edition2" sheetId="12" r:id="rId25"/>
-    <sheet name="RiskAssessmentNo" sheetId="13" r:id="rId26"/>
+    <sheet name="Competitive Creation Modal" sheetId="29" r:id="rId17"/>
+    <sheet name="Creation Second Modal for App" sheetId="25" r:id="rId18"/>
+    <sheet name="Creation Second Modal FA" sheetId="24" r:id="rId19"/>
+    <sheet name="Creation Second Modal1" sheetId="14" r:id="rId20"/>
+    <sheet name="Creation Second Modal3" sheetId="17" r:id="rId21"/>
+    <sheet name="Creation Second Modal4" sheetId="18" r:id="rId22"/>
+    <sheet name="Creation of Second Modal" sheetId="15" r:id="rId23"/>
+    <sheet name="EnterReview" sheetId="9" r:id="rId24"/>
+    <sheet name="Pre-Application Modal" sheetId="11" r:id="rId25"/>
+    <sheet name="Edition2" sheetId="12" r:id="rId26"/>
+    <sheet name="RiskAssessmentNo" sheetId="13" r:id="rId27"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -50,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="662" uniqueCount="90">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -1445,7 +1446,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B029D8-A57A-4DED-8831-111F395CEFC2}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
@@ -1606,6 +1607,13 @@
         <v>33</v>
       </c>
     </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B15" s="6"/>
+      <c r="C15" s="4"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B16" s="6"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -1613,6 +1621,197 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49F19099-5305-442F-9CD7-4437184F40A1}">
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.140625" customWidth="1"/>
+    <col min="2" max="2" width="36.7109375" customWidth="1"/>
+    <col min="3" max="3" width="37.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>78</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C16" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A5EA066-8BD7-4F60-A549-8DF4B566C85E}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1769,7 +1968,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68EBF6E6-8687-4CE1-8BB6-330DEC350611}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1875,174 +2074,6 @@
       </c>
       <c r="C9" t="s">
         <v>33</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
-        <v>39</v>
-      </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>37</v>
-      </c>
-      <c r="C12" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>41</v>
-      </c>
-      <c r="C13" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>42</v>
-      </c>
-      <c r="C14" t="s">
-        <v>33</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B71B207-7F71-4F84-BC32-C3056B8DABA1}">
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>36</v>
-      </c>
-      <c r="C7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>38</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -2165,6 +2196,174 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B71B207-7F71-4F84-BC32-C3056B8DABA1}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFE25EE6-66F5-4951-9D0C-F6559D035D9C}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2322,7 +2521,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B83C7FC7-2A18-436E-A373-D289D769241C}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2491,7 +2690,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{471A3BD1-3EAB-4C67-9345-90730B6A7403}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2659,7 +2858,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A836B93B-2094-42BE-9D92-A2EB5434CB28}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2707,7 +2906,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB402F88-9436-4279-8D3B-028474BBC575}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2875,7 +3074,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61C91C76-2A92-4FAB-8589-A8F89F7DC3A0}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2915,7 +3114,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF72FB96-7C2F-4711-BDC9-46D87BC44E74}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Updated for execution test
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New LWC\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{817DBBDD-AF66-4BE3-B3CC-95CE1CD3EB53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8840F943-9552-4D17-B462-AFC8F66380F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="795" firstSheet="37" activeTab="42" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="795" firstSheet="14" activeTab="14" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement_Admin" sheetId="44" r:id="rId1"/>
@@ -460,9 +460,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -500,7 +500,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -606,7 +606,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -748,7 +748,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>

</xml_diff>

<commit_message>
set up for demo branch and registartion flow added
</commit_message>
<xml_diff>
--- a/src/main/resources/Announcement_Field_Values.xlsx
+++ b/src/main/resources/Announcement_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Cleanup_Projects\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Santosh J\REI Projects\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2C2F1FF-15A3-431C-821E-7860E648E1C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{205304D1-4AA2-4EDD-87ED-1882212786C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="795" firstSheet="34" activeTab="35" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="795" firstSheet="8" activeTab="9" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement_Admin" sheetId="44" r:id="rId1"/>
@@ -972,10 +972,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07BD69C2-DB57-4C60-8DCC-FB9C43CEE49A}">
   <sheetPr codeName="Sheet39"/>
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="1" max="1" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.36328125" customWidth="1"/>
     <col min="3" max="3" width="43" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1036,10 +1036,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9C8260A-2B08-45B2-91C9-3D139644FA31}">
   <sheetPr codeName="Sheet9"/>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="1" max="1" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.36328125" customWidth="1"/>
     <col min="3" max="3" width="59" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1100,9 +1100,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{801045D0-434D-4772-B50B-BAD32ADFCC6D}">
   <sheetPr codeName="Sheet10"/>
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="33.6640625" customWidth="1"/>
+    <col min="1" max="1" width="33.6328125" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="55" customWidth="1"/>
   </cols>
@@ -1160,10 +1160,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{312DC3EE-E575-46F9-A9B5-EB471905BC17}">
   <sheetPr codeName="Sheet11"/>
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" customWidth="1"/>
-    <col min="3" max="3" width="65.6640625" customWidth="1"/>
+    <col min="2" max="2" width="29.453125" customWidth="1"/>
+    <col min="3" max="3" width="65.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1220,10 +1220,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{628A250B-2421-4501-B6A1-3551362D1E63}">
   <sheetPr codeName="Sheet12"/>
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="31.33203125" customWidth="1"/>
-    <col min="3" max="3" width="46.5546875" customWidth="1"/>
+    <col min="2" max="2" width="31.36328125" customWidth="1"/>
+    <col min="3" max="3" width="46.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1279,9 +1279,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67385A93-9DB4-418E-B977-B594C234D617}">
   <sheetPr codeName="Sheet13"/>
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="44.6640625" customWidth="1"/>
+    <col min="2" max="2" width="44.6328125" customWidth="1"/>
     <col min="3" max="3" width="38" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1339,10 +1339,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32F7954A-D9CB-47FE-8043-C26DF94F149F}">
   <sheetPr codeName="Sheet14"/>
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="52.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="52.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1397,10 +1397,10 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CB0B370-5042-41B9-A8EC-24D7CD1FD99D}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="27.33203125" customWidth="1"/>
-    <col min="3" max="3" width="59.5546875" customWidth="1"/>
+    <col min="2" max="2" width="27.36328125" customWidth="1"/>
+    <col min="3" max="3" width="59.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1456,10 +1456,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C81AF588-AABE-4434-A649-BE45CA5F0598}">
   <sheetPr codeName="Sheet15"/>
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="1" max="1" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.36328125" customWidth="1"/>
     <col min="3" max="3" width="43" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1517,10 +1517,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F5A36B1-BCE1-494C-9FF2-9E81EB69D145}">
   <sheetPr codeName="Sheet16"/>
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="1" max="1" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.36328125" customWidth="1"/>
     <col min="3" max="3" width="43" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1578,11 +1578,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E513E26F-ED03-4E26-8F3C-BE6B3D3F87CC}">
   <sheetPr codeName="Sheet17"/>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="44.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1696,11 +1696,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EABAA4BE-5C71-4904-8238-AC9EDD6FB8A9}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="30.44140625" customWidth="1"/>
-    <col min="2" max="2" width="26.33203125" customWidth="1"/>
-    <col min="3" max="3" width="62.33203125" customWidth="1"/>
+    <col min="1" max="1" width="30.453125" customWidth="1"/>
+    <col min="2" max="2" width="26.36328125" customWidth="1"/>
+    <col min="3" max="3" width="62.36328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1756,9 +1756,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5419849D-2139-4751-9485-A00468AD6907}">
   <sheetPr codeName="Sheet18"/>
   <dimension ref="A1:G14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
@@ -1924,9 +1924,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FF67A45-0B54-4944-9B39-F82B26EF60B6}">
   <sheetPr codeName="Sheet19"/>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
@@ -2039,10 +2039,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F105F821-5E53-4FD8-9F07-CF97205700C1}">
   <sheetPr codeName="Sheet20"/>
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="32.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2187,10 +2187,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC101BFC-1550-4137-B012-E4749B310065}">
   <sheetPr codeName="Sheet21"/>
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2323,11 +2323,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896B5C7-9641-468E-8213-95D0BE0FBE7C}">
   <sheetPr codeName="Sheet22"/>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2372,10 +2372,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
   <sheetPr codeName="Sheet23"/>
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2454,11 +2454,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5689EA4D-03A7-4B71-84BE-6001E09A3DD3}">
   <sheetPr codeName="Sheet24"/>
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="13.44140625" customWidth="1"/>
-    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.33203125" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" customWidth="1"/>
+    <col min="2" max="2" width="30.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.36328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2624,10 +2624,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{366DB7B4-C63A-47E9-A3AB-3A17CFD5CE09}">
   <sheetPr codeName="Sheet25"/>
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2793,10 +2793,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AA6F82E-C68B-45AF-AB19-9A11877150E6}">
   <sheetPr codeName="Sheet26"/>
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2963,11 +2963,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F8CA48C-2A2F-44CF-A1AF-B3B67AA99C99}">
   <sheetPr codeName="Sheet27"/>
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -3134,11 +3134,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FA2A7B2-CA79-4318-86DD-0D44A813A1C3}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="58.6640625" customWidth="1"/>
+    <col min="1" max="1" width="7.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="58.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -3199,9 +3199,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B029D8-A57A-4DED-8831-111F395CEFC2}">
   <sheetPr codeName="Sheet28"/>
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3368,10 +3368,10 @@
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A74E35D3-1628-483E-8955-C1943DBA1691}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="28.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -3537,9 +3537,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A5EA066-8BD7-4F60-A549-8DF4B566C85E}">
   <sheetPr codeName="Sheet29"/>
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3706,9 +3706,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68EBF6E6-8687-4CE1-8BB6-330DEC350611}">
   <sheetPr codeName="Sheet30"/>
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3875,9 +3875,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B71B207-7F71-4F84-BC32-C3056B8DABA1}">
   <sheetPr codeName="Sheet31"/>
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4043,10 +4043,10 @@
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60D5F1C4-68E1-4C20-A92E-5B34A98159BC}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="42.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -4157,10 +4157,10 @@
 <file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2441CEEE-9CD5-4C8F-8478-53A90F75A93B}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="43.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="43.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -4270,10 +4270,10 @@
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC020E3F-9A4F-4380-8601-0ACA44065B96}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="43.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="43.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -4383,9 +4383,9 @@
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B323604F-295C-41B0-98DA-4297355A795E}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="3" max="3" width="43.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="43.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -4495,7 +4495,7 @@
 <file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC944E47-2270-4A88-AAB7-CDD2A686FB82}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -4605,9 +4605,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98DDFB63-7F7A-4DD0-8939-BEB21ABE0A0F}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4774,7 +4774,7 @@
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{444B0433-D92D-4AC8-A1E6-731472E8EAC0}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
@@ -4883,10 +4883,10 @@
 <file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65CC1C52-FEAB-4BC2-90D1-ACBAA592B349}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="43.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="43.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -4996,11 +4996,11 @@
 <file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9A61549-7A09-42D8-B378-89BCE97801B7}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -5099,10 +5099,10 @@
 <file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E30494C-3CF8-41CD-A871-52E96E60A3C8}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -5157,11 +5157,11 @@
 <file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0FD23B6-DB16-49EB-89A8-BE20588C8004}">
   <dimension ref="A1:C35"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -5558,10 +5558,10 @@
 <file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BD489B9-7D28-4D0A-968C-65911560FD33}">
   <dimension ref="A1:C34"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="31.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -5946,11 +5946,11 @@
 <file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE27BAAE-CFD6-49EB-92C1-4C1E4D395BD6}">
   <dimension ref="A1:C34"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="23.44140625" customWidth="1"/>
-    <col min="2" max="2" width="23.88671875" customWidth="1"/>
-    <col min="3" max="3" width="40.44140625" customWidth="1"/>
+    <col min="1" max="1" width="23.453125" customWidth="1"/>
+    <col min="2" max="2" width="23.90625" customWidth="1"/>
+    <col min="3" max="3" width="40.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -6335,7 +6335,7 @@
 <file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E2A0686-D278-4AC7-8259-F9DC9C794771}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6344,10 +6344,10 @@
 <file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8878618-1E7E-452C-8F3E-1824580DC013}">
   <dimension ref="A1:C35"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="31.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -6743,10 +6743,10 @@
 <file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3322F882-9846-42CB-AFD8-EF8376DE9FFF}">
   <dimension ref="A1:C29"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="31.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -7077,9 +7077,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AFE106B-11CB-4012-8BB8-CD21B4581FD8}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="37" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
@@ -7233,10 +7233,10 @@
 <file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7ABB0E19-6DD3-4701-AD61-80C76D45A082}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="27" customWidth="1"/>
-    <col min="3" max="3" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="21.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -7391,10 +7391,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFE25EE6-66F5-4951-9D0C-F6559D035D9C}">
   <sheetPr codeName="Sheet32"/>
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="14.5546875" customWidth="1"/>
-    <col min="2" max="2" width="31.6640625" customWidth="1"/>
+    <col min="1" max="1" width="14.54296875" customWidth="1"/>
+    <col min="2" max="2" width="31.6328125" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7561,11 +7561,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B83C7FC7-2A18-436E-A373-D289D769241C}">
   <sheetPr codeName="Sheet33"/>
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" customWidth="1"/>
-    <col min="2" max="2" width="24.44140625" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" customWidth="1"/>
+    <col min="1" max="1" width="12.54296875" customWidth="1"/>
+    <col min="2" max="2" width="24.453125" customWidth="1"/>
+    <col min="3" max="3" width="15.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -7731,9 +7731,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{471A3BD1-3EAB-4C67-9345-90730B6A7403}">
   <sheetPr codeName="Sheet34"/>
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7899,10 +7899,10 @@
 <file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B540E81-1FD2-4AA2-8DEE-8BFB8B274149}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="34.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.6328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7937,10 +7937,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A836B93B-2094-42BE-9D92-A2EB5434CB28}">
   <sheetPr codeName="Sheet35"/>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -7986,9 +7986,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB402F88-9436-4279-8D3B-028474BBC575}">
   <sheetPr codeName="Sheet36"/>
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -8155,9 +8155,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61C91C76-2A92-4FAB-8589-A8F89F7DC3A0}">
   <sheetPr codeName="Sheet37"/>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" bestFit="1" customWidth="1"/>
   </cols>
@@ -8196,10 +8196,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF72FB96-7C2F-4711-BDC9-46D87BC44E74}">
   <sheetPr codeName="Sheet38"/>
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="1" max="1" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.36328125" customWidth="1"/>
     <col min="3" max="3" width="43" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -8366,10 +8366,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE354EA7-EF61-4CF6-8FD9-4C0F8CF01A30}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="1" max="1" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.36328125" customWidth="1"/>
     <col min="3" max="3" width="43" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -8430,11 +8430,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FC5EB7D-13BF-4B5E-895C-F5B651828B55}">
   <sheetPr codeName="Sheet6"/>
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="30.44140625" customWidth="1"/>
-    <col min="2" max="2" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="62.33203125" customWidth="1"/>
+    <col min="1" max="1" width="30.453125" customWidth="1"/>
+    <col min="2" max="2" width="27.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="62.36328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -8490,10 +8490,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C170638-B62F-4953-B95A-AF6F648592AA}">
   <sheetPr codeName="Sheet7"/>
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="59.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="59.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -8549,10 +8549,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27E9C587-3A78-4B4A-BCAE-07DA844DEBEA}">
   <sheetPr codeName="Sheet8"/>
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="53.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">

</xml_diff>